<commit_message>
feat: add Supabase authentication integration, recruiter sign-in modal, and docs
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -1083,7 +1083,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>Arjun’s standout strength is designing stateful multi-agent systems with LangGraph, supported by a robust Python FastAPI backend. His portfolio highlights 13 relevant AI repositories, including an embeddings-based retrieval pipeline using LangChain and PostgreSQL. While his GitHub activity shows sustained building over three years, the absence of Redis or backend caching evidence remains a notable technical gap. Still, his focus on complex orchestration and RAG architectures makes him a strong fit for our high-volume AI infrastructure team.</t>
+          <t>At 81.5/100, Arjun Kumar stands out through strong public github footprint (veteran builder), complemented by automated testing / ci/cd pipeline. Plus observability and concurrency handling rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, AWS maps to AI 35.0 and Python 25.0 bands. GitHub profile: Veteran Builder (3.0 yrs on GitHub, 26 repos [24 original], 226 contributions in past year [0 commits], 2 stars). 13 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>Arunima’s portfolio reveals a sophisticated grasp of stateful multi-agent orchestration via LangGraph, a standout capability for complex AI workflows. Her backend architecture leverages Python, FastAPI, and PostgreSQL, demonstrating solid full-stack integration with Docker and cloud providers. However, the absence of a public GitHub profile hinders direct code review, while limited evidence of Redis caching or explicit pytest unit tests suggests a gap in production-readiness. This profile fits our SDE AI internship, requiring mentorship to bridge the delta between prototype complexity and rigorous, testable engineering standards.</t>
+          <t>Arunima Saha (75.5/100) impressed with advanced rag with hybrid search and reranking alongside ai evaluation pipeline (ragas/langsmith/trulens). Also notable: modern python backend framework (fastapi/django). Depth spans Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS (cloud 11.0/15, GitHub 0.0/10). Activity: No public GitHub profile provided. Interview focus should be no explicit testing (pytest/unit tests) mentioned, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>Abhinav’s portfolio reveals a seasoned builder with 3.4 years of consistent output, including 61 repositories and 4,315 contributions last year. His technical core is anchored in a modern Python backend using FastAPI, PostgreSQL, and Redis, complemented by sophisticated stateful multi-agent orchestration via LangGraph. This combination of robust API design and advanced RAG implementation demonstrates rare depth for an intern. With no major gaps identified, his proven engineering discipline and broad Azure experience make him an immediate, high-value addition to our AI infrastructure team.</t>
+          <t>Abhinav Mishra (73.5/100) impressed with observability and concurrency handling alongside stateful multi-agent orchestration (langgraph/crewai/autogen). Also notable: embeddings-based retrieval system. Depth spans Python, FastAPI, PostgreSQL, Redis, Azure, LangGraph (cloud 8.0/15, GitHub 10.0/10). Activity: Veteran Builder (3.4 yrs on GitHub, 61 repos [28 original], 4315 contributions in past year [0 commits, 1 PRs], 7 stars). 9 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>Jyandeep Baishya’s profile reveals a committed builder, evidenced by 45 repositories and 490 annual contributions. His technical foundation is solid, leveraging Python, FastAPI, and Redis to construct robust backend systems. He effectively integrates LangChain, LangGraph, and ChromaDB to deploy RAG pipelines and multi-agent workflows. While his GitHub history demonstrates consistent, original work, the absence of explicit testing frameworks like pytest remains a notable gap. This candidate is ready to contribute to our AI infrastructure, requiring mentorship to rigorize quality assurance practices during the internship.</t>
+          <t>Jyandeep Baishya (73.0/100) impressed with stateful multi-agent orchestration (langgraph/crewai/autogen) alongside vector database retrieval (chromadb/faiss/pinecone/qdrant). Also notable: async fastapi backend architecture. Depth spans Python, FastAPI, Redis, LangChain, LangGraph, RAG (cloud 8.0/15, GitHub 10.0/10). Activity: Veteran Builder (3.4 yrs on GitHub, 45 repos [29 original], 490 contributions in past year [0 commits], 1 stars). 7 relevant Python/AI repositories identified. Interview focus should be no explicit testing (pytest/unit tests) mentioned, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>Krishan’s four-year GitHub tenure reveals a builder’s mindset, anchored by two relevant Python/AI repositories. His strongest signal is an agentic workflow leveraging LangChain and OpenAI for function calling, paired with a robust embeddings-based retrieval system using PostgreSQL and Redis. While the stack is solid, the absence of explicit pytest unit tests hints at a need for rigorous engineering discipline. This gap, however, is exactly what our internship program targets, offering him the structured mentorship to refine his RAG pipelines into production-grade, testable code.</t>
+          <t>Krishan Kant scored 70.0/100 (AI 23.0/40, Python 25.0/30, Cloud 10.0/15, GitHub 9.0/10), led by strong public github footprint (veteran builder) and distributed task queues (celery/rabbitmq/kafka) Backed by observability and concurrency handling. Stack centers on Python, PostgreSQL, Redis, Docker. GitHub: Veteran Builder (4.0 yrs on GitHub, 21 repos [14 original], 21 contributions in past year [0 commits], 5 stars). 2 relevant Python/AI repositories identified. Watch-item: no explicit testing (pytest/unit tests) mentioned. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>Priyanshu Kumar (63.0/100) impressed with full stack capability (react/next.js/typescript) alongside strong public github footprint (veteran builder). Also notable: distributed task queues (celery/rabbitmq/kafka). Depth spans Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG (cloud 4.0/15, GitHub 7.5/10). Activity: Veteran Builder (3.3 yrs on GitHub, 13 repos [9 original], 5 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
+          <t>Priyanshu’s profile hinges on stateful multi-agent orchestration using LangGraph and vector retrieval via Pinecone. His Python and FastAPI work shows promise in RAG pipelines, leveraging LangChain embeddings for robust data handling. However, the absence of explicit testing frameworks like pytest is a notable gap for production readiness. Given his 3.3-year GitHub history with nine original repositories, he demonstrates consistent initiative. This foundation makes him a viable fit for an internship focused on refining agentic backend systems, provided mentorship addresses rigorous software engineering practices and caching strategies.</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="X20" s="3" t="inlineStr">
         <is>
-          <t>M Sai Kushith’s portfolio reveals a promising trajectory, anchored by one relevant Python/AI repository demonstrating RAG capabilities via LangChain and LangGraph. While the backend infrastructure is minimal, the integration of PostgreSQL suggests foundational database literacy. However, the 1.3-year GitHub history with only four total repositories indicates limited sustained engineering output. The absence of explicit testing practices or Redis caching remains a critical gap. Despite these shortcomings, the niche focus on retrieval systems warrants a junior internship to build robust backend discipline.</t>
+          <t>At 61.0/100, M Sai Kushith stands out through full stack capability (react/next.js/typescript), complemented by stateful multi-agent orchestration (langgraph/crewai/autogen). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, LangChain maps to AI 31.0 and Python 20.0 bands. GitHub profile: Active Builder (1.3 yrs on GitHub, 4 repos [4 original], 1 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="X35" s="3" t="inlineStr">
         <is>
-          <t>Agam, your portfolio demonstrates solid full-stack proficiency, particularly in building responsive interfaces with Next.js and managing state via React. However, we specifically require demonstrable experience with AI integration or agentic workflows to join this team. While your Python and FastAPI backend skills are strong, the absence of any RAG or LLM-driven project evidence means you haven’t met our core technical bar. To move forward, please highlight a specific project showcasing advanced AI implementation.</t>
+          <t>Screening result: Agam Jain ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, FastAPI, PostgreSQL, Redis, Docker) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="X40" s="3" t="inlineStr">
         <is>
-          <t>Kartikay’s portfolio highlights a solid grasp of frontend engineering, particularly with React and Next.js. However, the role demands robust Python backend experience, which is entirely absent from your stack. More critically, we require demonstrable AI or agentic project evidence, such as RAG implementations, which you haven’t provided. To move forward, please prepare a Python-based project showcasing autonomous agent workflows. This specific technical depth is non-negotiable for this internship track.</t>
+          <t>Screening result: Kartikay Sinha ineligible (0.0/100) — no evidence of python stack, no ai/agentic project evidence. Seen skills (Docker, React, Next.js, Typescript, Javascript) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="X47" s="3" t="inlineStr">
         <is>
-          <t>Your portfolio highlights strong proficiency in modern frontend frameworks like Next.js and TypeScript, showcasing solid engineering fundamentals. However, we specifically require demonstrated backend expertise in Python, which is entirely absent from your experience. Furthermore, there is no evidence of AI or agentic system development, a core requirement for this role. To be considered, you must showcase projects involving Python-based backend services and concrete implementations of RAG or autonomous agent architectures.</t>
+          <t>Shivam Raj does not advance (ineligible, 0.0/100). Core gap: no evidence of python stack, no ai/agentic project evidence. While Docker, Azure, React, Next.js, Typescript shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="X50" s="3" t="inlineStr">
         <is>
-          <t>Vishwas, your full-stack portfolio is solid, but the lack of AI integration is a hard stop. We specifically require evidence of agentic workflows or RAG implementation, which your Flask and React projects don't demonstrate. Your Python backend skills are a strong foundation, but they aren't enough on their own. To clear this bar, you need to showcase a project where you actively built or deployed an LLM-driven agent or retrieval system, not just standard CRUD operations.</t>
+          <t>Screening result: Vishwas Badiger ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Flask, React, Javascript, Node.Js) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="X51" s="3" t="inlineStr">
         <is>
-          <t>Your Django and PostgreSQL backend skills are solid, but we can’t move forward without concrete AI or agentic project evidence. The mandatory bar for this role requires demonstrated experience with RAG pipelines or autonomous agent frameworks, which your current portfolio lacks. To become competitive, build a distinct project showcasing LLM integration or agent orchestration. While your REST API and Docker experience shows good engineering fundamentals, the absence of AI-specific work prevents us from advancing your application further.</t>
+          <t>Screening result: Yuvaraj R ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Django, PostgreSQL, Docker, Rest Api) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update screening results output
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -711,7 +711,7 @@
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>At 94.5/100, V Sree Raghu Vardhan stands out through cloud infrastructure (aws/azure), complemented by full stack capability (react/next.js/typescript). Plus strong public github footprint (veteran builder) rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, Redis maps to AI 37.0 and Python 30.0 bands. GitHub profile: Veteran Builder (4.2 yrs on GitHub, 35 repos [24 original], 45 contributions in past year [0 commits]). 3 relevant Python/AI repositories identified. Growth edge to probe in interview: polishing production hardening.</t>
+          <t>With a 94.5 score, this candidate’s mastery of Stateful multi-agent orchestration and Vector database retrieval stands out. Their architecture leverages Python, FastAPI, and PostgreSQL, scaled via Docker and AWS. GitHub history shows 35 repos over four years, including three relevant Python/AI projects. Though recent contribution volume is low, the depth of original work is significant. No major gaps exist, making them an immediate fit for our SDE AI internship.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>Priyanshu’s profile hinges on stateful multi-agent orchestration using LangGraph and vector retrieval via Pinecone. His Python and FastAPI work shows promise in RAG pipelines, leveraging LangChain embeddings for robust data handling. However, the absence of explicit testing frameworks like pytest is a notable gap for production readiness. Given his 3.3-year GitHub history with nine original repositories, he demonstrates consistent initiative. This foundation makes him a viable fit for an internship focused on refining agentic backend systems, provided mentorship addresses rigorous software engineering practices and caching strategies.</t>
+          <t>Priyanshu Kumar (63.0/100) impressed with full stack capability (react/next.js/typescript) alongside strong public github footprint (veteran builder). Also notable: distributed task queues (celery/rabbitmq/kafka). Depth spans Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG (cloud 4.0/15, GitHub 7.5/10). Activity: Veteran Builder (3.3 yrs on GitHub, 13 repos [9 original], 5 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="X37" s="3" t="inlineStr">
         <is>
-          <t>Gayathri Palraj was marked ineligible at 0.0/100 due to no ai/agentic project evidence. Background shows Python, React, Typescript, Javascript, Node.Js, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
+          <t>Gayathri, your proficiency in TypeScript and React is evident, yet your portfolio lacks the critical agentic or RAG implementation required for this role. While your Python and Node.js fundamentals are solid, we specifically need tangible evidence of AI backend development or multi-step reasoning systems. To clear this bar, please submit a project demonstrating a functional AI agent, such as a tool-using assistant or a retrieval-augmented generation pipeline, to prove your readiness for our advanced AI stack.</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="X46" s="3" t="inlineStr">
         <is>
-          <t>Programming Language Python does not advance (ineligible, 0.0/100). Core gap: no ai/agentic project evidence. While Python, React, Javascript, GIT, SQL shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
+          <t>Your portfolio highlights solid frontend work with React and Javascript, demonstrating clear technical proficiency. However, you lack the mandatory AI/agentic project evidence required for this role. Specifically, there is no proof of backend Python expertise or experience building RAG systems. To clear this bar, please showcase a project where you utilized Python to engineer an intelligent, autonomous agent or retrieval-augmented generation pipeline.</t>
         </is>
       </c>
     </row>

</xml_diff>